<commit_message>
schedule and venue details for the conference. You can also find the list of sponsors and exhibitors, and the conference poster here.        </div>        <div class="stat-row">          <div><div class="stat-n">9</div><div class="stat-l">KeyNote <br> Sessions</div></div>          <div><div class="stat-n">3</div><div class="stat-l">Workshops</div></div>          <div><div class="stat-n">4</div><div class="stat-l">Tracks</div></div>          <div><div class="stat-n">3</div><div class="stat-l">Days</div></div>          <div><div class="stat-n">300+</div><div class="stat-l">Delegates</div></div>        </div>      </div>      """, unsafe_allow_html=True)
</commit_message>
<xml_diff>
--- a/conference_data.xlsx
+++ b/conference_data.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Attendees" sheetId="1" r:id="rId1"/>
-    <sheet name="Schedule" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
+    <sheet name="Schedule" sheetId="3" r:id="rId2"/>
+    <sheet name="Schedule1" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -104,9 +104,6 @@
     <t>Day 1</t>
   </si>
   <si>
-    <t>04.06.2026</t>
-  </si>
-  <si>
     <t>08:15 - 09:15</t>
   </si>
   <si>
@@ -414,12 +411,18 @@
   </si>
   <si>
     <t>Valedictory</t>
+  </si>
+  <si>
+    <t>01.06.2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -471,7 +474,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -481,6 +484,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -819,94 +823,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" customWidth="1"/>
-    <col min="3" max="3" width="21.85546875" customWidth="1"/>
-    <col min="4" max="4" width="24.42578125" customWidth="1"/>
-    <col min="6" max="8" width="9.140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" s="1">
-        <v>0.375</v>
-      </c>
-      <c r="C2" s="1">
-        <v>0.4375</v>
-      </c>
-      <c r="D2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" s="1">
-        <v>0.41666666666666702</v>
-      </c>
-      <c r="C3" s="1">
-        <v>0.47916666666666702</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="1">
-        <v>0.45833333333333298</v>
-      </c>
-      <c r="C4" s="1">
-        <v>0.52083333333333304</v>
-      </c>
-      <c r="D4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B5" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="C5" s="1">
-        <v>0.5625</v>
-      </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -948,11 +864,11 @@
       <c r="A2" t="s">
         <v>26</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="C2" t="s">
         <v>27</v>
-      </c>
-      <c r="C2" t="s">
-        <v>28</v>
       </c>
       <c r="D2" s="2">
         <v>0.34375</v>
@@ -961,21 +877,21 @@
         <v>0.38541666666666669</v>
       </c>
       <c r="F2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H2" t="s">
         <v>29</v>
-      </c>
-      <c r="H2" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>26</v>
       </c>
-      <c r="B3" t="s">
-        <v>27</v>
+      <c r="B3" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="C3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D3" s="2">
         <v>0.38541666666666669</v>
@@ -984,47 +900,47 @@
         <v>0.41666666666666669</v>
       </c>
       <c r="F3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H3" t="s">
         <v>32</v>
-      </c>
-      <c r="H3" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>26</v>
       </c>
-      <c r="B4" t="s">
-        <v>27</v>
+      <c r="B4" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D4" s="2">
-        <v>0.38541666666666669</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="E4" s="2">
         <v>0.4513888888888889</v>
       </c>
       <c r="F4" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>36</v>
-      </c>
       <c r="H4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>26</v>
       </c>
-      <c r="B5" t="s">
-        <v>27</v>
+      <c r="B5" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="C5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D5" s="2">
         <v>0.4513888888888889</v>
@@ -1033,21 +949,21 @@
         <v>0.45833333333333331</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>26</v>
       </c>
-      <c r="B6" t="s">
-        <v>27</v>
+      <c r="B6" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="C6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D6" s="2">
         <v>0.46527777777777773</v>
@@ -1056,24 +972,24 @@
         <v>0.5</v>
       </c>
       <c r="F6" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G6" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="G6" s="3" t="s">
-        <v>41</v>
-      </c>
       <c r="H6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>26</v>
       </c>
-      <c r="B7" t="s">
-        <v>27</v>
+      <c r="B7" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="C7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D7" s="2">
         <v>0.5</v>
@@ -1085,18 +1001,18 @@
         <v>20</v>
       </c>
       <c r="H7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>26</v>
       </c>
-      <c r="B8" t="s">
-        <v>27</v>
+      <c r="B8" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="C8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D8" s="2">
         <v>0.55208333333333337</v>
@@ -1105,21 +1021,21 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="F8" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H8" t="s">
         <v>45</v>
-      </c>
-      <c r="H8" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>26</v>
       </c>
-      <c r="B9" t="s">
-        <v>27</v>
+      <c r="B9" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="C9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D9" s="2">
         <v>0.55208333333333337</v>
@@ -1128,21 +1044,21 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="F9" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="H9" t="s">
         <v>47</v>
-      </c>
-      <c r="H9" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>26</v>
       </c>
-      <c r="B10" t="s">
-        <v>27</v>
+      <c r="B10" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="C10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D10" s="2">
         <v>0.55208333333333337</v>
@@ -1151,21 +1067,21 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="F10" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H10" t="s">
         <v>49</v>
-      </c>
-      <c r="H10" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>26</v>
       </c>
-      <c r="B11" t="s">
-        <v>27</v>
+      <c r="B11" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="C11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D11" s="2">
         <v>0.55208333333333337</v>
@@ -1174,21 +1090,21 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="F11" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H11" t="s">
         <v>51</v>
-      </c>
-      <c r="H11" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>26</v>
       </c>
-      <c r="B12" t="s">
-        <v>27</v>
+      <c r="B12" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="C12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D12" s="2">
         <v>0.55208333333333337</v>
@@ -1197,21 +1113,21 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="F12" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="H12" t="s">
         <v>53</v>
-      </c>
-      <c r="H12" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>26</v>
       </c>
-      <c r="B13" t="s">
-        <v>27</v>
+      <c r="B13" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="C13" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D13" s="2">
         <v>0.55208333333333337</v>
@@ -1220,21 +1136,21 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="F13" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H13" t="s">
         <v>55</v>
-      </c>
-      <c r="H13" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>26</v>
       </c>
-      <c r="B14" t="s">
-        <v>27</v>
+      <c r="B14" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="C14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D14" s="2">
         <v>0.55208333333333337</v>
@@ -1243,21 +1159,21 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="F14" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H14" t="s">
         <v>57</v>
-      </c>
-      <c r="H14" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>26</v>
       </c>
-      <c r="B15" t="s">
-        <v>27</v>
+      <c r="B15" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="C15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D15" s="2">
         <v>0.64583333333333337</v>
@@ -1266,24 +1182,24 @@
         <v>0.68055555555555547</v>
       </c>
       <c r="F15" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G15" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="G15" s="3" t="s">
-        <v>61</v>
-      </c>
       <c r="H15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>26</v>
       </c>
-      <c r="B16" t="s">
-        <v>27</v>
+      <c r="B16" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="C16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D16" s="2">
         <v>0.68055555555555547</v>
@@ -1292,21 +1208,21 @@
         <v>0.6875</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>26</v>
       </c>
-      <c r="B17" t="s">
-        <v>27</v>
+      <c r="B17" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="C17" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D17" s="2">
         <v>0.6875</v>
@@ -1315,21 +1231,21 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>26</v>
       </c>
-      <c r="B18" t="s">
-        <v>27</v>
+      <c r="B18" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="C18" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D18" s="2">
         <v>0.70833333333333337</v>
@@ -1338,21 +1254,21 @@
         <v>0.77083333333333337</v>
       </c>
       <c r="F18" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H18" t="s">
         <v>67</v>
-      </c>
-      <c r="H18" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>26</v>
       </c>
-      <c r="B19" t="s">
-        <v>27</v>
+      <c r="B19" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="C19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D19" s="2">
         <v>0.77083333333333337</v>
@@ -1361,21 +1277,21 @@
         <v>0.8125</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H19" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>70</v>
+      </c>
+      <c r="B20" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>72</v>
-      </c>
-      <c r="C20" t="s">
-        <v>73</v>
       </c>
       <c r="D20" s="2">
         <v>0.375</v>
@@ -1384,24 +1300,24 @@
         <v>0.40972222222222227</v>
       </c>
       <c r="F20" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="G20" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="G20" s="3" t="s">
-        <v>75</v>
-      </c>
       <c r="H20" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>70</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B21" t="s">
-        <v>72</v>
-      </c>
       <c r="C21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D21" s="2">
         <v>0.40972222222222227</v>
@@ -1410,24 +1326,24 @@
         <v>0.44444444444444442</v>
       </c>
       <c r="F21" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="G21" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="G21" s="3" t="s">
-        <v>78</v>
-      </c>
       <c r="H21" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>70</v>
+      </c>
+      <c r="B22" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B22" t="s">
-        <v>72</v>
-      </c>
       <c r="C22" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D22" s="2">
         <v>0.44444444444444442</v>
@@ -1436,21 +1352,21 @@
         <v>0.4513888888888889</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H22" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>70</v>
+      </c>
+      <c r="B23" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B23" t="s">
-        <v>72</v>
-      </c>
       <c r="C23" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D23" s="2">
         <v>0.4513888888888889</v>
@@ -1459,21 +1375,21 @@
         <v>0.53472222222222221</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H23" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>70</v>
+      </c>
+      <c r="B24" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B24" t="s">
-        <v>72</v>
-      </c>
       <c r="C24" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D24" s="2">
         <v>0.53472222222222221</v>
@@ -1485,18 +1401,18 @@
         <v>20</v>
       </c>
       <c r="H24" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>70</v>
+      </c>
+      <c r="B25" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B25" t="s">
-        <v>72</v>
-      </c>
       <c r="C25" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D25" s="2">
         <v>0.56944444444444442</v>
@@ -1505,24 +1421,24 @@
         <v>0.60416666666666663</v>
       </c>
       <c r="F25" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="G25" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="G25" s="3" t="s">
-        <v>85</v>
-      </c>
       <c r="H25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>70</v>
+      </c>
+      <c r="B26" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B26" t="s">
-        <v>72</v>
-      </c>
       <c r="C26" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D26" s="2">
         <v>0.60416666666666663</v>
@@ -1531,21 +1447,21 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="F26" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="H26" t="s">
         <v>87</v>
-      </c>
-      <c r="H26" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>70</v>
+      </c>
+      <c r="B27" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B27" t="s">
-        <v>72</v>
-      </c>
       <c r="C27" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D27" s="2">
         <v>0.60416666666666663</v>
@@ -1554,21 +1470,21 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="F27" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="H27" t="s">
         <v>89</v>
-      </c>
-      <c r="H27" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>70</v>
+      </c>
+      <c r="B28" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B28" t="s">
-        <v>72</v>
-      </c>
       <c r="C28" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D28" s="2">
         <v>0.60416666666666663</v>
@@ -1577,21 +1493,21 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="F28" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="H28" t="s">
         <v>91</v>
-      </c>
-      <c r="H28" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>70</v>
+      </c>
+      <c r="B29" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B29" t="s">
-        <v>72</v>
-      </c>
       <c r="C29" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D29" s="2">
         <v>0.66666666666666663</v>
@@ -1600,21 +1516,21 @@
         <v>0.67361111111111116</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H29" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>70</v>
+      </c>
+      <c r="B30" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B30" t="s">
-        <v>72</v>
-      </c>
       <c r="C30" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D30" s="2">
         <v>0.67361111111111116</v>
@@ -1623,21 +1539,21 @@
         <v>0.77083333333333337</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H30" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>70</v>
+      </c>
+      <c r="B31" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B31" t="s">
-        <v>72</v>
-      </c>
       <c r="C31" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D31" s="2">
         <v>0.67361111111111116</v>
@@ -1646,21 +1562,21 @@
         <v>0.77083333333333337</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H31" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>70</v>
+      </c>
+      <c r="B32" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B32" t="s">
-        <v>72</v>
-      </c>
       <c r="C32" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D32" s="2">
         <v>0.79166666666666663</v>
@@ -1669,21 +1585,21 @@
         <v>0.85416666666666663</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H32" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>98</v>
+      </c>
+      <c r="B33" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B33" t="s">
-        <v>100</v>
-      </c>
       <c r="C33" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D33" s="2">
         <v>0.375</v>
@@ -1692,24 +1608,24 @@
         <v>0.40972222222222227</v>
       </c>
       <c r="F33" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G33" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="G33" s="3" t="s">
-        <v>102</v>
-      </c>
       <c r="H33" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>98</v>
+      </c>
+      <c r="B34" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B34" t="s">
-        <v>100</v>
-      </c>
       <c r="C34" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D34" s="2">
         <v>0.40972222222222227</v>
@@ -1718,24 +1634,24 @@
         <v>0.44444444444444442</v>
       </c>
       <c r="F34" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="G34" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="G34" s="3" t="s">
-        <v>104</v>
-      </c>
       <c r="H34" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>98</v>
+      </c>
+      <c r="B35" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B35" t="s">
-        <v>100</v>
-      </c>
       <c r="C35" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D35" s="2">
         <v>0.44444444444444442</v>
@@ -1744,21 +1660,21 @@
         <v>0.4513888888888889</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H35" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>98</v>
+      </c>
+      <c r="B36" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B36" t="s">
-        <v>100</v>
-      </c>
       <c r="C36" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D36" s="2">
         <v>0.4513888888888889</v>
@@ -1767,21 +1683,21 @@
         <v>0.53472222222222221</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H36" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>98</v>
+      </c>
+      <c r="B37" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B37" t="s">
-        <v>100</v>
-      </c>
       <c r="C37" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D37" s="2">
         <v>0.4513888888888889</v>
@@ -1790,21 +1706,21 @@
         <v>0.53472222222222221</v>
       </c>
       <c r="F37" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="H37" t="s">
         <v>106</v>
-      </c>
-      <c r="H37" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>98</v>
+      </c>
+      <c r="B38" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B38" t="s">
-        <v>100</v>
-      </c>
       <c r="C38" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D38" s="2">
         <v>0.4513888888888889</v>
@@ -1813,21 +1729,21 @@
         <v>0.53472222222222221</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H38" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>98</v>
+      </c>
+      <c r="B39" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B39" t="s">
-        <v>100</v>
-      </c>
       <c r="C39" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D39" s="2">
         <v>0.4513888888888889</v>
@@ -1836,21 +1752,21 @@
         <v>0.53472222222222221</v>
       </c>
       <c r="F39" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="H39" t="s">
         <v>109</v>
-      </c>
-      <c r="H39" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>98</v>
+      </c>
+      <c r="B40" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B40" t="s">
-        <v>100</v>
-      </c>
       <c r="C40" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D40" s="2">
         <v>0.4513888888888889</v>
@@ -1859,21 +1775,21 @@
         <v>0.53472222222222221</v>
       </c>
       <c r="F40" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="H40" t="s">
         <v>111</v>
-      </c>
-      <c r="H40" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>98</v>
+      </c>
+      <c r="B41" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B41" t="s">
-        <v>100</v>
-      </c>
       <c r="C41" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D41" s="2">
         <v>0.4513888888888889</v>
@@ -1882,21 +1798,21 @@
         <v>0.53472222222222221</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H41" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>98</v>
+      </c>
+      <c r="B42" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B42" t="s">
-        <v>100</v>
-      </c>
       <c r="C42" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D42" s="2">
         <v>0.4513888888888889</v>
@@ -1905,21 +1821,21 @@
         <v>0.53472222222222221</v>
       </c>
       <c r="F42" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="H42" t="s">
         <v>114</v>
-      </c>
-      <c r="H42" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>98</v>
+      </c>
+      <c r="B43" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B43" t="s">
-        <v>100</v>
-      </c>
       <c r="C43" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D43" s="2">
         <v>0.52083333333333337</v>
@@ -1931,18 +1847,18 @@
         <v>20</v>
       </c>
       <c r="H43" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>98</v>
+      </c>
+      <c r="B44" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B44" t="s">
-        <v>100</v>
-      </c>
       <c r="C44" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D44" s="2">
         <v>0.54166666666666663</v>
@@ -1951,21 +1867,21 @@
         <v>0.625</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H44" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>98</v>
+      </c>
+      <c r="B45" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B45" t="s">
-        <v>100</v>
-      </c>
       <c r="C45" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D45" s="2">
         <v>0.54166666666666663</v>
@@ -1974,21 +1890,21 @@
         <v>0.625</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H45" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>98</v>
+      </c>
+      <c r="B46" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B46" t="s">
-        <v>100</v>
-      </c>
       <c r="C46" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D46" s="2">
         <v>0.54166666666666663</v>
@@ -1997,21 +1913,21 @@
         <v>0.625</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H46" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>98</v>
+      </c>
+      <c r="B47" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B47" t="s">
-        <v>100</v>
-      </c>
       <c r="C47" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D47" s="2">
         <v>0.54166666666666663</v>
@@ -2020,21 +1936,21 @@
         <v>0.625</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H47" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>98</v>
+      </c>
+      <c r="B48" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B48" t="s">
-        <v>100</v>
-      </c>
       <c r="C48" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D48" s="2">
         <v>0.54166666666666663</v>
@@ -2043,21 +1959,21 @@
         <v>0.625</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H48" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>98</v>
+      </c>
+      <c r="B49" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B49" t="s">
-        <v>100</v>
-      </c>
       <c r="C49" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D49" s="2">
         <v>0.54166666666666663</v>
@@ -2066,21 +1982,21 @@
         <v>0.625</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H49" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>98</v>
+      </c>
+      <c r="B50" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B50" t="s">
-        <v>100</v>
-      </c>
       <c r="C50" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D50" s="2">
         <v>0.54166666666666663</v>
@@ -2089,21 +2005,21 @@
         <v>0.625</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H50" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>98</v>
+      </c>
+      <c r="B51" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B51" t="s">
-        <v>100</v>
-      </c>
       <c r="C51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D51" s="2">
         <v>0.625</v>
@@ -2112,21 +2028,21 @@
         <v>0.63194444444444442</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H51" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>98</v>
+      </c>
+      <c r="B52" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B52" t="s">
-        <v>100</v>
-      </c>
       <c r="C52" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D52" s="2">
         <v>0.63194444444444442</v>
@@ -2135,24 +2051,24 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="F52" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="G52" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="G52" s="3" t="s">
-        <v>128</v>
-      </c>
       <c r="H52" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>98</v>
+      </c>
+      <c r="B53" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B53" t="s">
-        <v>100</v>
-      </c>
       <c r="C53" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D53" s="2">
         <v>0.66666666666666663</v>
@@ -2161,13 +2077,102 @@
         <v>0.70138888888888884</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H53" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" customWidth="1"/>
+    <col min="3" max="3" width="21.85546875" customWidth="1"/>
+    <col min="4" max="4" width="24.42578125" customWidth="1"/>
+    <col min="6" max="8" width="9.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="1">
+        <v>0.375</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.4375</v>
+      </c>
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="1">
+        <v>0.41666666666666702</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0.47916666666666702</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="1">
+        <v>0.45833333333333298</v>
+      </c>
+      <c r="C4" s="1">
+        <v>0.52083333333333304</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0.5625</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
new feature of maps added to the app.py file
</commit_message>
<xml_diff>
--- a/conference_data.xlsx
+++ b/conference_data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="133">
   <si>
     <t>Conference_ID</t>
   </si>
@@ -104,6 +104,9 @@
     <t>Day 1</t>
   </si>
   <si>
+    <t>04.06.2026</t>
+  </si>
+  <si>
     <t>08:15 - 09:15</t>
   </si>
   <si>
@@ -414,6 +417,9 @@
   </si>
   <si>
     <t>01.06.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin Council Hall </t>
   </si>
 </sst>
 </file>
@@ -799,7 +805,7 @@
         <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -865,10 +871,10 @@
         <v>26</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D2" s="2">
         <v>0.34375</v>
@@ -877,10 +883,10 @@
         <v>0.38541666666666669</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -888,10 +894,10 @@
         <v>26</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D3" s="2">
         <v>0.38541666666666669</v>
@@ -900,10 +906,10 @@
         <v>0.41666666666666669</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -911,10 +917,10 @@
         <v>26</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D4" s="2">
         <v>0.41666666666666669</v>
@@ -923,13 +929,13 @@
         <v>0.4513888888888889</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -937,10 +943,10 @@
         <v>26</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D5" s="2">
         <v>0.4513888888888889</v>
@@ -949,10 +955,10 @@
         <v>0.45833333333333331</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -960,10 +966,10 @@
         <v>26</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D6" s="2">
         <v>0.46527777777777773</v>
@@ -972,13 +978,13 @@
         <v>0.5</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -986,10 +992,10 @@
         <v>26</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D7" s="2">
         <v>0.5</v>
@@ -1001,7 +1007,7 @@
         <v>20</v>
       </c>
       <c r="H7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1009,10 +1015,10 @@
         <v>26</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D8" s="2">
         <v>0.55208333333333337</v>
@@ -1021,10 +1027,10 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1032,10 +1038,10 @@
         <v>26</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D9" s="2">
         <v>0.55208333333333337</v>
@@ -1044,10 +1050,10 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="H9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1055,10 +1061,10 @@
         <v>26</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D10" s="2">
         <v>0.55208333333333337</v>
@@ -1067,10 +1073,10 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -1078,10 +1084,10 @@
         <v>26</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D11" s="2">
         <v>0.55208333333333337</v>
@@ -1090,10 +1096,10 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -1101,10 +1107,10 @@
         <v>26</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C12" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D12" s="2">
         <v>0.55208333333333337</v>
@@ -1113,10 +1119,10 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1124,10 +1130,10 @@
         <v>26</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D13" s="2">
         <v>0.55208333333333337</v>
@@ -1136,10 +1142,10 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -1147,10 +1153,10 @@
         <v>26</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C14" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D14" s="2">
         <v>0.55208333333333337</v>
@@ -1159,10 +1165,10 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -1170,10 +1176,10 @@
         <v>26</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>130</v>
+        <v>27</v>
       </c>
       <c r="C15" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D15" s="2">
         <v>0.64583333333333337</v>
@@ -1182,13 +1188,13 @@
         <v>0.68055555555555547</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H15" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -1196,10 +1202,10 @@
         <v>26</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C16" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D16" s="2">
         <v>0.68055555555555547</v>
@@ -1208,10 +1214,10 @@
         <v>0.6875</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H16" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -1219,10 +1225,10 @@
         <v>26</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C17" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D17" s="2">
         <v>0.6875</v>
@@ -1231,10 +1237,10 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H17" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -1242,10 +1248,10 @@
         <v>26</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C18" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D18" s="2">
         <v>0.70833333333333337</v>
@@ -1254,10 +1260,10 @@
         <v>0.77083333333333337</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -1265,10 +1271,10 @@
         <v>26</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C19" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D19" s="2">
         <v>0.77083333333333337</v>
@@ -1277,21 +1283,21 @@
         <v>0.8125</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H19" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C20" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D20" s="2">
         <v>0.375</v>
@@ -1300,24 +1306,24 @@
         <v>0.40972222222222227</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H20" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C21" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D21" s="2">
         <v>0.40972222222222227</v>
@@ -1326,24 +1332,24 @@
         <v>0.44444444444444442</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H21" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C22" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D22" s="2">
         <v>0.44444444444444442</v>
@@ -1352,21 +1358,21 @@
         <v>0.4513888888888889</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H22" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C23" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D23" s="2">
         <v>0.4513888888888889</v>
@@ -1375,21 +1381,21 @@
         <v>0.53472222222222221</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H23" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C24" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D24" s="2">
         <v>0.53472222222222221</v>
@@ -1401,18 +1407,18 @@
         <v>20</v>
       </c>
       <c r="H24" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C25" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D25" s="2">
         <v>0.56944444444444442</v>
@@ -1421,24 +1427,24 @@
         <v>0.60416666666666663</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H25" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C26" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D26" s="2">
         <v>0.60416666666666663</v>
@@ -1447,21 +1453,21 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H26" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C27" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D27" s="2">
         <v>0.60416666666666663</v>
@@ -1470,21 +1476,21 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H27" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>71</v>
+        <v>131</v>
       </c>
       <c r="C28" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D28" s="2">
         <v>0.60416666666666663</v>
@@ -1493,21 +1499,21 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H28" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C29" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D29" s="2">
         <v>0.66666666666666663</v>
@@ -1516,21 +1522,21 @@
         <v>0.67361111111111116</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H29" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C30" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D30" s="2">
         <v>0.67361111111111116</v>
@@ -1539,21 +1545,21 @@
         <v>0.77083333333333337</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C31" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D31" s="2">
         <v>0.67361111111111116</v>
@@ -1562,21 +1568,21 @@
         <v>0.77083333333333337</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H31" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C32" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D32" s="2">
         <v>0.79166666666666663</v>
@@ -1585,21 +1591,21 @@
         <v>0.85416666666666663</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H32" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C33" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D33" s="2">
         <v>0.375</v>
@@ -1608,24 +1614,24 @@
         <v>0.40972222222222227</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H33" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C34" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D34" s="2">
         <v>0.40972222222222227</v>
@@ -1634,24 +1640,24 @@
         <v>0.44444444444444442</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H34" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C35" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D35" s="2">
         <v>0.44444444444444442</v>
@@ -1660,21 +1666,21 @@
         <v>0.4513888888888889</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H35" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C36" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D36" s="2">
         <v>0.4513888888888889</v>
@@ -1683,21 +1689,21 @@
         <v>0.53472222222222221</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H36" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C37" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D37" s="2">
         <v>0.4513888888888889</v>
@@ -1706,21 +1712,21 @@
         <v>0.53472222222222221</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H37" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C38" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D38" s="2">
         <v>0.4513888888888889</v>
@@ -1729,21 +1735,21 @@
         <v>0.53472222222222221</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H38" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C39" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D39" s="2">
         <v>0.4513888888888889</v>
@@ -1752,21 +1758,21 @@
         <v>0.53472222222222221</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H39" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C40" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D40" s="2">
         <v>0.4513888888888889</v>
@@ -1775,21 +1781,21 @@
         <v>0.53472222222222221</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H40" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C41" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D41" s="2">
         <v>0.4513888888888889</v>
@@ -1798,21 +1804,21 @@
         <v>0.53472222222222221</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H41" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C42" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D42" s="2">
         <v>0.4513888888888889</v>
@@ -1821,21 +1827,21 @@
         <v>0.53472222222222221</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H42" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C43" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D43" s="2">
         <v>0.52083333333333337</v>
@@ -1847,18 +1853,18 @@
         <v>20</v>
       </c>
       <c r="H43" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C44" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D44" s="2">
         <v>0.54166666666666663</v>
@@ -1867,21 +1873,21 @@
         <v>0.625</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H44" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C45" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D45" s="2">
         <v>0.54166666666666663</v>
@@ -1890,21 +1896,21 @@
         <v>0.625</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H45" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C46" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D46" s="2">
         <v>0.54166666666666663</v>
@@ -1913,21 +1919,21 @@
         <v>0.625</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H46" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C47" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D47" s="2">
         <v>0.54166666666666663</v>
@@ -1936,21 +1942,21 @@
         <v>0.625</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H47" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C48" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D48" s="2">
         <v>0.54166666666666663</v>
@@ -1959,21 +1965,21 @@
         <v>0.625</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H48" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C49" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D49" s="2">
         <v>0.54166666666666663</v>
@@ -1982,21 +1988,21 @@
         <v>0.625</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H49" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C50" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D50" s="2">
         <v>0.54166666666666663</v>
@@ -2005,21 +2011,21 @@
         <v>0.625</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H50" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C51" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D51" s="2">
         <v>0.625</v>
@@ -2028,21 +2034,21 @@
         <v>0.63194444444444442</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H51" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C52" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D52" s="2">
         <v>0.63194444444444442</v>
@@ -2051,24 +2057,24 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H52" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C53" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D53" s="2">
         <v>0.66666666666666663</v>
@@ -2077,10 +2083,10 @@
         <v>0.70138888888888884</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H53" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>